<commit_message>
Update lmbench docs and ratio tables
</commit_message>
<xml_diff>
--- a/docs/n90-kvm-host/lmbench-N10-4config-mean.xlsx
+++ b/docs/n90-kvm-host/lmbench-N10-4config-mean.xlsx
@@ -2555,7 +2555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2592,306 +2592,318 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>results/n90-day3/n90-{kvmoff,nvhe,vhe,pkvm}-noLSM-full-cpu0.csv</t>
+          <t>results/n90-day3-host/n90-{kvmoff,nvhe,vhe,pkvm}-noLSM-full-cpu0.csv</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>每个配置 iter 数</t>
+          <t>lat_mmap 高精度覆盖</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>N=10</t>
+          <t>results/precise-mmap/*.log 覆盖 0.5/1/2/4/8/16/64 MB 行</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>CPU 频率</t>
+          <t>每个配置 iter 数</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>锁 1900 MHz, governor=performance</t>
+          <t>N=10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>LSM 栈</t>
+          <t>CPU 频率</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>capability,kycp（无 ksaf/bpf/audit）</t>
+          <t>锁 1900 MHz, governor=performance</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>THP</t>
+          <t>LSM 栈</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>never</t>
+          <t>capability,kycp（无 ksaf/bpf/audit）</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>ASLR</t>
+          <t>THP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>never</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>绑核</t>
+          <t>ASLR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>cpu0 (taskset -c 0)</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>lmbench config</t>
+          <t>绑核</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CONFIG.host（全套 BENCHMARK_*=YES）</t>
+          <t>cpu0 (taskset -c 0)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
+          <t>lmbench config</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CONFIG.host（全套 BENCHMARK_*=YES）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
           <t>噪声抑制</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>72 项系统 + 12 项用户 systemd 服务 mask，桌面 multi-user.target</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Sheet 说明：</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Highlights</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>论文表 (Sci China Inf Sci) 30+ 项 + lat_mmap/mem hierarchy/bw 重点</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  All metrics</t>
+          <t xml:space="preserve">  Highlights</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>全部 684 项 (bench, variant) 中位 + MAD% + 5 个跨配置 Δ%</t>
+          <t>论文表 (Sci China Inf Sci) 30+ 项 + lat_mmap/mem hierarchy/bw 重点</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">  All metrics</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>全部 684 项 (bench, variant) 均值 + RSD% + 5 个跨配置 Δ%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Per-iter raw</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>论文重点项的 10 个 iter 单值（用于自己重新算 stat）</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>论文重点项的 10 个 iter 单值 + 均值/RSD%</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Δ% 颜色编码（方向 × 强度）：</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  方向（按指标单位判断）：</t>
-        </is>
-      </c>
+      <c r="A21" s="12" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    单位 us / ns（延迟）</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>负 Δ% → 更快 → 绿；正 Δ% → 更慢 → 红</t>
+          <t xml:space="preserve">  方向（按指标单位判断）：</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    单位 MB/s（带宽）</t>
+          <t xml:space="preserve">    单位 us / ns（延迟）</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>正 Δ% → 更高 → 绿；负 Δ% → 更低 → 红</t>
+          <t>负 Δ% → 更快 → 绿；正 Δ% → 更慢 → 红</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">    单位 MB/s（带宽）</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>正 Δ% → 更高 → 绿；负 Δ% → 更低 → 红</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">    单位 pages（TLB）</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>正 Δ% → 更大 → 绿；负 Δ% → 更小 → 红</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  强度：</t>
-        </is>
-      </c>
+      <c r="A26" s="12" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    |Δ| &gt; 10%</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>深色 + 粗体（显著差异）</t>
+          <t xml:space="preserve">  强度：</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    5% &lt; |Δ| ≤ 10%</t>
+          <t xml:space="preserve">    |Δ| &gt; 10%</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>中等色</t>
+          <t>深色 + 粗体（显著差异）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    2% &lt; |Δ| ≤ 5%</t>
+          <t xml:space="preserve">    5% &lt; |Δ| ≤ 10%</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>浅色</t>
+          <t>中等色</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">    2% &lt; |Δ| ≤ 5%</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>浅色</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">    |Δ| ≤ 2%</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>黑色（在 MAD 噪声范围内，不算差异）</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>关键 finding：</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. host syscall fastpath 4 模式无差（≤ 1%）</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2. CPU 算术 4 模式绝对相等（sanity ✓）</t>
+          <t xml:space="preserve">  1. host syscall fastpath 4 模式无差（≤ 1%）</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. pkvm 在 lat_mmap 大段比其它 3 模式慢 +15-42%（stage-2 表维护）</t>
+          <t xml:space="preserve">  2. CPU 算术 4 模式绝对相等（sanity ✓）</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. host EL2 (vhe) vs host EL1 (kvmoff/nvhe) 无可观测性能差</t>
+          <t xml:space="preserve">  3. pkvm 在 lat_mmap 大段比其它 3 模式慢 +15-42%（stage-2 表维护）</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. host EL2 (vhe) vs host EL1 (kvmoff/nvhe) 无可观测性能差</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  5. TLB / cache 层级 / bw_mem 4 模式相等</t>
         </is>
@@ -41474,10 +41486,10 @@
         <v>0.1028</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>0.1028</v>
+        <v>0.10283</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>0</v>
+        <v>0.0469751912418226</v>
       </c>
     </row>
     <row r="3">
@@ -41519,10 +41531,10 @@
         <v>0.1029</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>0.1029</v>
+        <v>0.10309</v>
       </c>
       <c r="O3" s="5" t="n">
-        <v>0.04859086491739692</v>
+        <v>0.4673383551161669</v>
       </c>
     </row>
     <row r="4">
@@ -41564,10 +41576,10 @@
         <v>0.1028</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>0.1028</v>
+        <v>0.10283</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>0</v>
+        <v>0.0469751912418226</v>
       </c>
     </row>
     <row r="5">
@@ -41609,10 +41621,10 @@
         <v>0.1028</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>0.10285</v>
+        <v>0.10296</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>0.04861448711716231</v>
+        <v>0.3581796603454866</v>
       </c>
     </row>
     <row r="6">
@@ -41662,10 +41674,10 @@
         <v>1.4902</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>1.49515</v>
+        <v>1.49775</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>0.1070126743136096</v>
+        <v>0.6564177602188723</v>
       </c>
     </row>
     <row r="7">
@@ -41707,10 +41719,10 @@
         <v>1.4974</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>1.4898</v>
+        <v>1.49077</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>0.134246207544637</v>
+        <v>0.3539784555452379</v>
       </c>
     </row>
     <row r="8">
@@ -41752,10 +41764,10 @@
         <v>1.4925</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>1.49125</v>
+        <v>1.48974</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>0.1274098910310077</v>
+        <v>0.2655257256535879</v>
       </c>
     </row>
     <row r="9">
@@ -41797,10 +41809,10 @@
         <v>1.4971</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>1.49715</v>
+        <v>1.4971</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>0.0333967872290723</v>
+        <v>0.1280591707928533</v>
       </c>
     </row>
     <row r="10">
@@ -41850,10 +41862,10 @@
         <v>136.1351</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>136.1903</v>
+        <v>136.35869</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>0.1921575912528417</v>
+        <v>0.5266146622990685</v>
       </c>
     </row>
     <row r="11">
@@ -41895,10 +41907,10 @@
         <v>136.5811</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>136.48105</v>
+        <v>136.57848</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>0.3575587966241256</v>
+        <v>0.6934784569723402</v>
       </c>
     </row>
     <row r="12">
@@ -41940,10 +41952,10 @@
         <v>135.9067</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>136.54695</v>
+        <v>136.49823</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>0.4258974660364125</v>
+        <v>0.5214378020025145</v>
       </c>
     </row>
     <row r="13">
@@ -41985,10 +41997,10 @@
         <v>138.9753</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>139.0679</v>
+        <v>139.11137</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>0.1334959397531676</v>
+        <v>0.311991577432128</v>
       </c>
     </row>
     <row r="14">
@@ -42038,10 +42050,10 @@
         <v>377.4286</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>377.3069</v>
+        <v>377.76289</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>0.5171387006174548</v>
+        <v>0.5381144693649166</v>
       </c>
     </row>
     <row r="15">
@@ -42083,10 +42095,10 @@
         <v>375.25</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>375.7431</v>
+        <v>376.70374</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>0.1839953947258189</v>
+        <v>0.6872284869235213</v>
       </c>
     </row>
     <row r="16">
@@ -42128,10 +42140,10 @@
         <v>376.4138</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>376.99815</v>
+        <v>377.62981</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>0.2520304144728507</v>
+        <v>0.5875661322616261</v>
       </c>
     </row>
     <row r="17">
@@ -42173,10 +42185,10 @@
         <v>384.8929</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>385.8393</v>
+        <v>386.32965</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>0.2175257937695772</v>
+        <v>0.5359410566398729</v>
       </c>
     </row>
     <row r="18">
@@ -42226,10 +42238,10 @@
         <v>796</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>796.7143</v>
+        <v>797.95715</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>0.2286139460531815</v>
+        <v>0.4321106035662554</v>
       </c>
     </row>
     <row r="19">
@@ -42271,10 +42283,10 @@
         <v>790.6667</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>792.7857</v>
+        <v>792.6881</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>0.2417614243041977</v>
+        <v>0.5280561624096</v>
       </c>
     </row>
     <row r="20">
@@ -42316,10 +42328,10 @@
         <v>797.4286</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>791.2856999999999</v>
+        <v>791.6642899999999</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>0.3069182218255632</v>
+        <v>0.5307262492683988</v>
       </c>
     </row>
     <row r="21">
@@ -42361,10 +42373,10 @@
         <v>812.5</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>807.60715</v>
+        <v>808.63571</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>0.3051359810274208</v>
+        <v>0.4837868103814547</v>
       </c>
     </row>
     <row r="22">
@@ -43166,10 +43178,10 @@
         <v>2.48</v>
       </c>
       <c r="N38" s="5" t="n">
-        <v>2.37</v>
+        <v>2.365</v>
       </c>
       <c r="O38" s="5" t="n">
-        <v>1.265822784810137</v>
+        <v>2.623609650315192</v>
       </c>
     </row>
     <row r="39">
@@ -43211,10 +43223,10 @@
         <v>2.35</v>
       </c>
       <c r="N39" s="5" t="n">
-        <v>2.38</v>
+        <v>2.383</v>
       </c>
       <c r="O39" s="5" t="n">
-        <v>1.260504201680664</v>
+        <v>2.755665660298173</v>
       </c>
     </row>
     <row r="40">
@@ -43256,10 +43268,10 @@
         <v>2.37</v>
       </c>
       <c r="N40" s="5" t="n">
-        <v>2.39</v>
+        <v>2.396</v>
       </c>
       <c r="O40" s="5" t="n">
-        <v>1.046025104602507</v>
+        <v>2.451053483087948</v>
       </c>
     </row>
     <row r="41">
@@ -43301,10 +43313,10 @@
         <v>2.3</v>
       </c>
       <c r="N41" s="5" t="n">
-        <v>2.365</v>
+        <v>2.369</v>
       </c>
       <c r="O41" s="5" t="n">
-        <v>1.268498942917558</v>
+        <v>2.307326668028281</v>
       </c>
     </row>
     <row r="42">
@@ -43354,10 +43366,10 @@
         <v>2.49</v>
       </c>
       <c r="N42" s="5" t="n">
-        <v>2.365</v>
+        <v>2.379</v>
       </c>
       <c r="O42" s="5" t="n">
-        <v>2.74841437632137</v>
+        <v>3.803545198941455</v>
       </c>
     </row>
     <row r="43">
@@ -43399,10 +43411,10 @@
         <v>2.38</v>
       </c>
       <c r="N43" s="5" t="n">
-        <v>2.38</v>
+        <v>2.382</v>
       </c>
       <c r="O43" s="5" t="n">
-        <v>2.310924369747906</v>
+        <v>3.397940153546308</v>
       </c>
     </row>
     <row r="44">
@@ -43444,10 +43456,10 @@
         <v>2.33</v>
       </c>
       <c r="N44" s="5" t="n">
-        <v>2.37</v>
+        <v>2.372</v>
       </c>
       <c r="O44" s="5" t="n">
-        <v>2.742616033755272</v>
+        <v>2.730738122876025</v>
       </c>
     </row>
     <row r="45">
@@ -43489,10 +43501,10 @@
         <v>2.34</v>
       </c>
       <c r="N45" s="5" t="n">
-        <v>2.385</v>
+        <v>2.388</v>
       </c>
       <c r="O45" s="5" t="n">
-        <v>1.04821802935011</v>
+        <v>1.551863998848388</v>
       </c>
     </row>
     <row r="46">
@@ -43542,10 +43554,10 @@
         <v>5.8</v>
       </c>
       <c r="N46" s="5" t="n">
-        <v>5.865</v>
+        <v>5.881</v>
       </c>
       <c r="O46" s="5" t="n">
-        <v>0.2557544757033345</v>
+        <v>0.9294434410064594</v>
       </c>
     </row>
     <row r="47">
@@ -43587,10 +43599,10 @@
         <v>5.88</v>
       </c>
       <c r="N47" s="5" t="n">
-        <v>5.859999999999999</v>
+        <v>5.858</v>
       </c>
       <c r="O47" s="5" t="n">
-        <v>0.8532423208191097</v>
+        <v>1.085028923323366</v>
       </c>
     </row>
     <row r="48">
@@ -43635,7 +43647,7 @@
         <v>5.85</v>
       </c>
       <c r="O48" s="5" t="n">
-        <v>0.7692307692307681</v>
+        <v>0.9045303627571258</v>
       </c>
     </row>
     <row r="49">
@@ -43677,10 +43689,10 @@
         <v>5.93</v>
       </c>
       <c r="N49" s="5" t="n">
-        <v>5.955</v>
+        <v>5.949</v>
       </c>
       <c r="O49" s="5" t="n">
-        <v>0.335852225020991</v>
+        <v>0.851425675967072</v>
       </c>
     </row>
     <row r="50">
@@ -43730,10 +43742,10 @@
         <v>6.01</v>
       </c>
       <c r="N50" s="5" t="n">
-        <v>5.985</v>
+        <v>5.988</v>
       </c>
       <c r="O50" s="5" t="n">
-        <v>0.3341687552213871</v>
+        <v>0.6624125932150281</v>
       </c>
     </row>
     <row r="51">
@@ -43775,10 +43787,10 @@
         <v>6.01</v>
       </c>
       <c r="N51" s="5" t="n">
-        <v>6</v>
+        <v>5.997</v>
       </c>
       <c r="O51" s="5" t="n">
-        <v>0.4166666666666652</v>
+        <v>0.5334264071595816</v>
       </c>
     </row>
     <row r="52">
@@ -43820,10 +43832,10 @@
         <v>5.97</v>
       </c>
       <c r="N52" s="5" t="n">
-        <v>6.025</v>
+        <v>6.023</v>
       </c>
       <c r="O52" s="5" t="n">
-        <v>0.3319502074688873</v>
+        <v>0.4764035467741949</v>
       </c>
     </row>
     <row r="53">
@@ -43865,10 +43877,10 @@
         <v>6.13</v>
       </c>
       <c r="N53" s="5" t="n">
-        <v>6.08</v>
+        <v>6.083</v>
       </c>
       <c r="O53" s="5" t="n">
-        <v>0.3289473684210456</v>
+        <v>0.5536990773880931</v>
       </c>
     </row>
     <row r="54">
@@ -43918,10 +43930,10 @@
         <v>5.5925</v>
       </c>
       <c r="N54" s="5" t="n">
-        <v>5.58645</v>
+        <v>5.57829</v>
       </c>
       <c r="O54" s="5" t="n">
-        <v>1.438301604775844</v>
+        <v>1.491697692327951</v>
       </c>
     </row>
     <row r="55">
@@ -43963,10 +43975,10 @@
         <v>5.6764</v>
       </c>
       <c r="N55" s="5" t="n">
-        <v>5.594849999999999</v>
+        <v>5.66702</v>
       </c>
       <c r="O55" s="5" t="n">
-        <v>1.987542114623249</v>
+        <v>3.990993708535578</v>
       </c>
     </row>
     <row r="56">
@@ -44008,10 +44020,10 @@
         <v>5.599</v>
       </c>
       <c r="N56" s="5" t="n">
-        <v>5.6151</v>
+        <v>5.72068</v>
       </c>
       <c r="O56" s="5" t="n">
-        <v>1.323217752132643</v>
+        <v>4.465451284455404</v>
       </c>
     </row>
     <row r="57">
@@ -44053,10 +44065,10 @@
         <v>5.5704</v>
       </c>
       <c r="N57" s="5" t="n">
-        <v>5.5435</v>
+        <v>5.53404</v>
       </c>
       <c r="O57" s="5" t="n">
-        <v>0.762153873906379</v>
+        <v>0.9818914504556892</v>
       </c>
     </row>
     <row r="58">
@@ -44106,10 +44118,10 @@
         <v>10.0752</v>
       </c>
       <c r="N58" s="5" t="n">
-        <v>10.3879</v>
+        <v>10.38556</v>
       </c>
       <c r="O58" s="5" t="n">
-        <v>3.063660605127118</v>
+        <v>5.624599611389928</v>
       </c>
     </row>
     <row r="59">
@@ -44151,10 +44163,10 @@
         <v>9.868399999999999</v>
       </c>
       <c r="N59" s="5" t="n">
-        <v>9.97405</v>
+        <v>10.17892</v>
       </c>
       <c r="O59" s="5" t="n">
-        <v>2.978729803840971</v>
+        <v>5.864299864370551</v>
       </c>
     </row>
     <row r="60">
@@ -44196,10 +44208,10 @@
         <v>9.811500000000001</v>
       </c>
       <c r="N60" s="5" t="n">
-        <v>9.860800000000001</v>
+        <v>10.02235</v>
       </c>
       <c r="O60" s="5" t="n">
-        <v>2.056628265455134</v>
+        <v>4.029953817517936</v>
       </c>
     </row>
     <row r="61">
@@ -44241,10 +44253,10 @@
         <v>9.8865</v>
       </c>
       <c r="N61" s="5" t="n">
-        <v>9.96495</v>
+        <v>10.05463</v>
       </c>
       <c r="O61" s="5" t="n">
-        <v>1.047672090677826</v>
+        <v>4.292032618421295</v>
       </c>
     </row>
     <row r="62">
@@ -44294,10 +44306,10 @@
         <v>15.9303</v>
       </c>
       <c r="N62" s="5" t="n">
-        <v>15.84425</v>
+        <v>15.86099</v>
       </c>
       <c r="O62" s="5" t="n">
-        <v>0.2351010618994231</v>
+        <v>0.457171279843709</v>
       </c>
     </row>
     <row r="63">
@@ -44339,10 +44351,10 @@
         <v>15.7625</v>
       </c>
       <c r="N63" s="5" t="n">
-        <v>16.0865</v>
+        <v>16.10631</v>
       </c>
       <c r="O63" s="5" t="n">
-        <v>0.5576104186740358</v>
+        <v>1.193728385758463</v>
       </c>
     </row>
     <row r="64">
@@ -44384,10 +44396,10 @@
         <v>16.0063</v>
       </c>
       <c r="N64" s="5" t="n">
-        <v>15.98055</v>
+        <v>16.01826</v>
       </c>
       <c r="O64" s="5" t="n">
-        <v>0.9552236938027758</v>
+        <v>1.397313254655398</v>
       </c>
     </row>
     <row r="65">
@@ -44429,10 +44441,10 @@
         <v>16.0819</v>
       </c>
       <c r="N65" s="5" t="n">
-        <v>15.9138</v>
+        <v>15.93167</v>
       </c>
       <c r="O65" s="5" t="n">
-        <v>0.1960562530633797</v>
+        <v>0.4367924389616558</v>
       </c>
     </row>
     <row r="66">
@@ -44482,10 +44494,10 @@
         <v>22.4927</v>
       </c>
       <c r="N66" s="5" t="n">
-        <v>22.48305</v>
+        <v>22.47696</v>
       </c>
       <c r="O66" s="5" t="n">
-        <v>0.2628646914008511</v>
+        <v>0.3176328041363534</v>
       </c>
     </row>
     <row r="67">
@@ -44527,10 +44539,10 @@
         <v>22.7462</v>
       </c>
       <c r="N67" s="5" t="n">
-        <v>22.6951</v>
+        <v>22.78191</v>
       </c>
       <c r="O67" s="5" t="n">
-        <v>1.007265885587638</v>
+        <v>1.285110526598172</v>
       </c>
     </row>
     <row r="68">
@@ -44572,10 +44584,10 @@
         <v>22.4296</v>
       </c>
       <c r="N68" s="5" t="n">
-        <v>22.64325</v>
+        <v>22.6276</v>
       </c>
       <c r="O68" s="5" t="n">
-        <v>0.7885352146887099</v>
+        <v>0.8282217281099095</v>
       </c>
     </row>
     <row r="69">
@@ -44617,10 +44629,10 @@
         <v>22.6377</v>
       </c>
       <c r="N69" s="5" t="n">
-        <v>22.65545</v>
+        <v>22.70049</v>
       </c>
       <c r="O69" s="5" t="n">
-        <v>0.2919827238037741</v>
+        <v>0.5792294556962231</v>
       </c>
     </row>
     <row r="70">
@@ -44670,10 +44682,10 @@
         <v>10826.6526</v>
       </c>
       <c r="N70" s="5" t="n">
-        <v>10713.5695</v>
+        <v>10717.01436</v>
       </c>
       <c r="O70" s="5" t="n">
-        <v>0.4455326490391585</v>
+        <v>0.5130517748062313</v>
       </c>
     </row>
     <row r="71">
@@ -44715,10 +44727,10 @@
         <v>10697.5985</v>
       </c>
       <c r="N71" s="5" t="n">
-        <v>10697.6112</v>
+        <v>10712.14154</v>
       </c>
       <c r="O71" s="5" t="n">
-        <v>0.2973476919781819</v>
+        <v>0.4253022667638796</v>
       </c>
     </row>
     <row r="72">
@@ -44760,10 +44772,10 @@
         <v>10745.6162</v>
       </c>
       <c r="N72" s="5" t="n">
-        <v>10705.5818</v>
+        <v>10715.27227</v>
       </c>
       <c r="O72" s="5" t="n">
-        <v>0.3713847667765223</v>
+        <v>0.3479552148812314</v>
       </c>
     </row>
     <row r="73">
@@ -44805,10 +44817,10 @@
         <v>10777.8707</v>
       </c>
       <c r="N73" s="5" t="n">
-        <v>10789.0136</v>
+        <v>10791.76851</v>
       </c>
       <c r="O73" s="5" t="n">
-        <v>0.3755510142280299</v>
+        <v>0.574947416946343</v>
       </c>
     </row>
     <row r="74">
@@ -44858,10 +44870,10 @@
         <v>93284</v>
       </c>
       <c r="N74" s="5" t="n">
-        <v>93501</v>
+        <v>93450.89999999999</v>
       </c>
       <c r="O74" s="5" t="n">
-        <v>0.1379664388616164</v>
+        <v>0.3227591612043804</v>
       </c>
     </row>
     <row r="75">
@@ -44903,10 +44915,10 @@
         <v>93707</v>
       </c>
       <c r="N75" s="5" t="n">
-        <v>93677.5</v>
+        <v>93564.10000000001</v>
       </c>
       <c r="O75" s="5" t="n">
-        <v>0.1675962744522431</v>
+        <v>0.46490988344681</v>
       </c>
     </row>
     <row r="76">
@@ -44948,10 +44960,10 @@
         <v>93654</v>
       </c>
       <c r="N76" s="5" t="n">
-        <v>93880.5</v>
+        <v>93838.3</v>
       </c>
       <c r="O76" s="5" t="n">
-        <v>0.2391337924276074</v>
+        <v>0.3339394862017426</v>
       </c>
     </row>
     <row r="77">
@@ -44993,10 +45005,10 @@
         <v>93168</v>
       </c>
       <c r="N77" s="5" t="n">
-        <v>92979</v>
+        <v>92892</v>
       </c>
       <c r="O77" s="5" t="n">
-        <v>0.1371277385216016</v>
+        <v>0.4666585214887897</v>
       </c>
     </row>
     <row r="78">
@@ -45046,10 +45058,10 @@
         <v>52968</v>
       </c>
       <c r="N78" s="5" t="n">
-        <v>52993</v>
+        <v>53025.4</v>
       </c>
       <c r="O78" s="5" t="n">
-        <v>0.09906968844941785</v>
+        <v>0.222021420275555</v>
       </c>
     </row>
     <row r="79">
@@ -45091,10 +45103,10 @@
         <v>52971</v>
       </c>
       <c r="N79" s="5" t="n">
-        <v>53094</v>
+        <v>53143.6</v>
       </c>
       <c r="O79" s="5" t="n">
-        <v>0.222247334915433</v>
+        <v>0.4420305594576099</v>
       </c>
     </row>
     <row r="80">
@@ -45136,10 +45148,10 @@
         <v>52939</v>
       </c>
       <c r="N80" s="5" t="n">
-        <v>53039.5</v>
+        <v>53115.9</v>
       </c>
       <c r="O80" s="5" t="n">
-        <v>0.2026791353613816</v>
+        <v>0.4548673112276939</v>
       </c>
     </row>
     <row r="81">
@@ -45181,10 +45193,10 @@
         <v>52617</v>
       </c>
       <c r="N81" s="5" t="n">
-        <v>52574.5</v>
+        <v>52584.9</v>
       </c>
       <c r="O81" s="5" t="n">
-        <v>0.2777011669155199</v>
+        <v>0.3404065651478686</v>
       </c>
     </row>
     <row r="82">
@@ -45234,10 +45246,10 @@
         <v>151557</v>
       </c>
       <c r="N82" s="5" t="n">
-        <v>151622.5</v>
+        <v>151799.6</v>
       </c>
       <c r="O82" s="5" t="n">
-        <v>0.4009958944088113</v>
+        <v>0.4212556514874579</v>
       </c>
     </row>
     <row r="83">
@@ -45279,10 +45291,10 @@
         <v>150987</v>
       </c>
       <c r="N83" s="5" t="n">
-        <v>153410.5</v>
+        <v>153158</v>
       </c>
       <c r="O83" s="5" t="n">
-        <v>0.3536263815058291</v>
+        <v>0.6797941187068148</v>
       </c>
     </row>
     <row r="84">
@@ -45324,10 +45336,10 @@
         <v>149759</v>
       </c>
       <c r="N84" s="5" t="n">
-        <v>151533.5</v>
+        <v>151650</v>
       </c>
       <c r="O84" s="5" t="n">
-        <v>0.3715350071106389</v>
+        <v>0.622154252152302</v>
       </c>
     </row>
     <row r="85">
@@ -45369,10 +45381,10 @@
         <v>151941</v>
       </c>
       <c r="N85" s="5" t="n">
-        <v>152021</v>
+        <v>151833.4</v>
       </c>
       <c r="O85" s="5" t="n">
-        <v>0.09571046105472271</v>
+        <v>0.7334029255507604</v>
       </c>
     </row>
     <row r="86">
@@ -45422,10 +45434,10 @@
         <v>89176</v>
       </c>
       <c r="N86" s="5" t="n">
-        <v>89628</v>
+        <v>89336.2</v>
       </c>
       <c r="O86" s="5" t="n">
-        <v>0.2828357209800509</v>
+        <v>0.6984098620074799</v>
       </c>
     </row>
     <row r="87">
@@ -45467,10 +45479,10 @@
         <v>89586</v>
       </c>
       <c r="N87" s="5" t="n">
-        <v>89977</v>
+        <v>89893.7</v>
       </c>
       <c r="O87" s="5" t="n">
-        <v>0.3584249308156529</v>
+        <v>0.6344343275245379</v>
       </c>
     </row>
     <row r="88">
@@ -45512,10 +45524,10 @@
         <v>89954</v>
       </c>
       <c r="N88" s="5" t="n">
-        <v>89947</v>
+        <v>89921.10000000001</v>
       </c>
       <c r="O88" s="5" t="n">
-        <v>0.1995619642678466</v>
+        <v>0.315824364330261</v>
       </c>
     </row>
     <row r="89">
@@ -45557,10 +45569,10 @@
         <v>88684</v>
       </c>
       <c r="N89" s="5" t="n">
-        <v>89429</v>
+        <v>89215.10000000001</v>
       </c>
       <c r="O89" s="5" t="n">
-        <v>0.188417627391562</v>
+        <v>0.4514606629782187</v>
       </c>
     </row>
     <row r="90">
@@ -45610,10 +45622,10 @@
         <v>0.1694</v>
       </c>
       <c r="N90" s="5" t="n">
-        <v>0.15905</v>
+        <v>0.16088</v>
       </c>
       <c r="O90" s="5" t="n">
-        <v>0.8173530336372182</v>
+        <v>3.292855918675945</v>
       </c>
     </row>
     <row r="91">
@@ -45655,10 +45667,10 @@
         <v>0.1629</v>
       </c>
       <c r="N91" s="5" t="n">
-        <v>0.15995</v>
+        <v>0.16036</v>
       </c>
       <c r="O91" s="5" t="n">
-        <v>0.9065332916536373</v>
+        <v>1.44019537278546</v>
       </c>
     </row>
     <row r="92">
@@ -45700,10 +45712,10 @@
         <v>0.1603</v>
       </c>
       <c r="N92" s="5" t="n">
-        <v>0.1602</v>
+        <v>0.16102</v>
       </c>
       <c r="O92" s="5" t="n">
-        <v>1.810237203495639</v>
+        <v>3.907768009430822</v>
       </c>
     </row>
     <row r="93">
@@ -45745,10 +45757,10 @@
         <v>0.1594</v>
       </c>
       <c r="N93" s="5" t="n">
-        <v>0.1594</v>
+        <v>0.15914</v>
       </c>
       <c r="O93" s="5" t="n">
-        <v>1.003764115432876</v>
+        <v>2.129531385818916</v>
       </c>
     </row>
     <row r="94">
@@ -45798,10 +45810,10 @@
         <v>0.2561</v>
       </c>
       <c r="N94" s="5" t="n">
-        <v>0.25445</v>
+        <v>0.25481</v>
       </c>
       <c r="O94" s="5" t="n">
-        <v>0.2947533896639814</v>
+        <v>0.61343000788448</v>
       </c>
     </row>
     <row r="95">
@@ -45843,10 +45855,10 @@
         <v>0.2579</v>
       </c>
       <c r="N95" s="5" t="n">
-        <v>0.2547</v>
+        <v>0.25497</v>
       </c>
       <c r="O95" s="5" t="n">
-        <v>0.2159403219474089</v>
+        <v>0.6640609321528245</v>
       </c>
     </row>
     <row r="96">
@@ -45888,10 +45900,10 @@
         <v>0.2581</v>
       </c>
       <c r="N96" s="5" t="n">
-        <v>0.25775</v>
+        <v>0.25722</v>
       </c>
       <c r="O96" s="5" t="n">
-        <v>0.2133850630456064</v>
+        <v>0.7854525329756943</v>
       </c>
     </row>
     <row r="97">
@@ -45933,10 +45945,10 @@
         <v>0.2627</v>
       </c>
       <c r="N97" s="5" t="n">
-        <v>0.25985</v>
+        <v>0.25987</v>
       </c>
       <c r="O97" s="5" t="n">
-        <v>0.2886280546469226</v>
+        <v>0.8444463495113552</v>
       </c>
     </row>
     <row r="98">
@@ -45986,10 +45998,10 @@
         <v>2.224</v>
       </c>
       <c r="N98" s="5" t="n">
-        <v>2.224</v>
+        <v>2.2238</v>
       </c>
       <c r="O98" s="5" t="n">
-        <v>0</v>
+        <v>0.01896020421602324</v>
       </c>
     </row>
     <row r="99">
@@ -46031,10 +46043,10 @@
         <v>2.224</v>
       </c>
       <c r="N99" s="5" t="n">
-        <v>2.224</v>
+        <v>2.2238</v>
       </c>
       <c r="O99" s="5" t="n">
-        <v>0</v>
+        <v>0.01896020421602324</v>
       </c>
     </row>
     <row r="100">
@@ -46076,10 +46088,10 @@
         <v>2.224</v>
       </c>
       <c r="N100" s="5" t="n">
-        <v>2.224</v>
+        <v>2.2239</v>
       </c>
       <c r="O100" s="5" t="n">
-        <v>0</v>
+        <v>0.01421951373789035</v>
       </c>
     </row>
     <row r="101">
@@ -46121,10 +46133,10 @@
         <v>2.224</v>
       </c>
       <c r="N101" s="5" t="n">
-        <v>2.224</v>
+        <v>2.2237</v>
       </c>
       <c r="O101" s="5" t="n">
-        <v>0</v>
+        <v>0.02172261957727253</v>
       </c>
     </row>
     <row r="102">
@@ -46174,10 +46186,10 @@
         <v>3.961</v>
       </c>
       <c r="N102" s="5" t="n">
-        <v>3.9705</v>
+        <v>3.9753</v>
       </c>
       <c r="O102" s="5" t="n">
-        <v>0.2770431935524579</v>
+        <v>0.6771775678373261</v>
       </c>
     </row>
     <row r="103">
@@ -46219,10 +46231,10 @@
         <v>3.984</v>
       </c>
       <c r="N103" s="5" t="n">
-        <v>3.9625</v>
+        <v>3.9524</v>
       </c>
       <c r="O103" s="5" t="n">
-        <v>0.4921135646687603</v>
+        <v>0.8732193476947568</v>
       </c>
     </row>
     <row r="104">
@@ -46264,10 +46276,10 @@
         <v>3.947</v>
       </c>
       <c r="N104" s="5" t="n">
-        <v>3.9405</v>
+        <v>3.9451</v>
       </c>
       <c r="O104" s="5" t="n">
-        <v>0.1776424311635609</v>
+        <v>0.9360398254214028</v>
       </c>
     </row>
     <row r="105">
@@ -46309,10 +46321,10 @@
         <v>3.993</v>
       </c>
       <c r="N105" s="5" t="n">
-        <v>3.9295</v>
+        <v>3.9401</v>
       </c>
       <c r="O105" s="5" t="n">
-        <v>0.5344191372948188</v>
+        <v>0.7529372198715252</v>
       </c>
     </row>
     <row r="106">
@@ -46362,10 +46374,10 @@
         <v>4.44</v>
       </c>
       <c r="N106" s="5" t="n">
-        <v>4.436999999999999</v>
+        <v>4.4365</v>
       </c>
       <c r="O106" s="5" t="n">
-        <v>0.1014198782961299</v>
+        <v>0.1473283861236549</v>
       </c>
     </row>
     <row r="107">
@@ -46407,10 +46419,10 @@
         <v>4.437</v>
       </c>
       <c r="N107" s="5" t="n">
-        <v>4.436500000000001</v>
+        <v>4.4363</v>
       </c>
       <c r="O107" s="5" t="n">
-        <v>0.07889101769412456</v>
+        <v>0.1052195972105006</v>
       </c>
     </row>
     <row r="108">
@@ -46455,7 +46467,7 @@
         <v>4.433</v>
       </c>
       <c r="O108" s="5" t="n">
-        <v>0.09023234829686451</v>
+        <v>0.1637081063018047</v>
       </c>
     </row>
     <row r="109">
@@ -46497,10 +46509,10 @@
         <v>4.432</v>
       </c>
       <c r="N109" s="5" t="n">
-        <v>4.435</v>
+        <v>4.4335</v>
       </c>
       <c r="O109" s="5" t="n">
-        <v>0.09019165727170243</v>
+        <v>0.1577992696651641</v>
       </c>
     </row>
     <row r="110">
@@ -46550,10 +46562,10 @@
         <v>10.35</v>
       </c>
       <c r="N110" s="5" t="n">
-        <v>10.815</v>
+        <v>11.2029</v>
       </c>
       <c r="O110" s="5" t="n">
-        <v>6.389274156264462</v>
+        <v>8.930149629526476</v>
       </c>
     </row>
     <row r="111">
@@ -46595,10 +46607,10 @@
         <v>10.02</v>
       </c>
       <c r="N111" s="5" t="n">
-        <v>11.41</v>
+        <v>11.2763</v>
       </c>
       <c r="O111" s="5" t="n">
-        <v>9.36897458369851</v>
+        <v>10.62239232925671</v>
       </c>
     </row>
     <row r="112">
@@ -46640,10 +46652,10 @@
         <v>12.631</v>
       </c>
       <c r="N112" s="5" t="n">
-        <v>12.447</v>
+        <v>11.9612</v>
       </c>
       <c r="O112" s="5" t="n">
-        <v>1.442114565758825</v>
+        <v>6.907604470517708</v>
       </c>
     </row>
     <row r="113">
@@ -46685,10 +46697,10 @@
         <v>12.474</v>
       </c>
       <c r="N113" s="5" t="n">
-        <v>12.123</v>
+        <v>11.6002</v>
       </c>
       <c r="O113" s="5" t="n">
-        <v>3.650086612224688</v>
+        <v>9.213961634588374</v>
       </c>
     </row>
     <row r="114">
@@ -46738,10 +46750,10 @@
         <v>10.19</v>
       </c>
       <c r="N114" s="5" t="n">
-        <v>10.357</v>
+        <v>10.3814</v>
       </c>
       <c r="O114" s="5" t="n">
-        <v>1.602780728010045</v>
+        <v>2.313677782437181</v>
       </c>
     </row>
     <row r="115">
@@ -46783,10 +46795,10 @@
         <v>10.641</v>
       </c>
       <c r="N115" s="5" t="n">
-        <v>10.241</v>
+        <v>10.302</v>
       </c>
       <c r="O115" s="5" t="n">
-        <v>1.821111219607457</v>
+        <v>2.095781280849246</v>
       </c>
     </row>
     <row r="116">
@@ -46828,10 +46840,10 @@
         <v>10.274</v>
       </c>
       <c r="N116" s="5" t="n">
-        <v>10.781</v>
+        <v>10.7839</v>
       </c>
       <c r="O116" s="5" t="n">
-        <v>3.158334106298113</v>
+        <v>3.534918087062341</v>
       </c>
     </row>
     <row r="117">
@@ -46873,10 +46885,10 @@
         <v>10.479</v>
       </c>
       <c r="N117" s="5" t="n">
-        <v>10.3445</v>
+        <v>10.411</v>
       </c>
       <c r="O117" s="5" t="n">
-        <v>1.416211513364586</v>
+        <v>1.955454434402476</v>
       </c>
     </row>
     <row r="118">
@@ -46926,10 +46938,10 @@
         <v>186.426</v>
       </c>
       <c r="N118" s="5" t="n">
-        <v>185.2325</v>
+        <v>182.2089</v>
       </c>
       <c r="O118" s="5" t="n">
-        <v>0.583860823559568</v>
+        <v>3.387335384634264</v>
       </c>
     </row>
     <row r="119">
@@ -46971,10 +46983,10 @@
         <v>184.506</v>
       </c>
       <c r="N119" s="5" t="n">
-        <v>185.045</v>
+        <v>181.1044</v>
       </c>
       <c r="O119" s="5" t="n">
-        <v>0.5482450214812526</v>
+        <v>4.254596262633656</v>
       </c>
     </row>
     <row r="120">
@@ -47016,10 +47028,10 @@
         <v>176.568</v>
       </c>
       <c r="N120" s="5" t="n">
-        <v>185.428</v>
+        <v>181.2069</v>
       </c>
       <c r="O120" s="5" t="n">
-        <v>0.3206096166706196</v>
+        <v>4.70844903943322</v>
       </c>
     </row>
     <row r="121">
@@ -47061,10 +47073,10 @@
         <v>178.793</v>
       </c>
       <c r="N121" s="5" t="n">
-        <v>191.7295</v>
+        <v>188.1345</v>
       </c>
       <c r="O121" s="5" t="n">
-        <v>0.2959899233034016</v>
+        <v>4.62574877276804</v>
       </c>
     </row>
     <row r="122">
@@ -47114,10 +47126,10 @@
         <v>113.05</v>
       </c>
       <c r="N122" s="5" t="n">
-        <v>112.5445</v>
+        <v>112.5996</v>
       </c>
       <c r="O122" s="5" t="n">
-        <v>0.3198734722709679</v>
+        <v>0.3963576785312238</v>
       </c>
     </row>
     <row r="123">
@@ -47159,10 +47171,10 @@
         <v>112.614</v>
       </c>
       <c r="N123" s="5" t="n">
-        <v>112.6005</v>
+        <v>112.6825</v>
       </c>
       <c r="O123" s="5" t="n">
-        <v>0.0706035941225928</v>
+        <v>0.2751045754367952</v>
       </c>
     </row>
     <row r="124">
@@ -47204,10 +47216,10 @@
         <v>112.335</v>
       </c>
       <c r="N124" s="5" t="n">
-        <v>112.325</v>
+        <v>112.374</v>
       </c>
       <c r="O124" s="5" t="n">
-        <v>0.0832405964834176</v>
+        <v>0.1764692903179884</v>
       </c>
     </row>
     <row r="125">
@@ -47249,10 +47261,10 @@
         <v>119.813</v>
       </c>
       <c r="N125" s="5" t="n">
-        <v>119.595</v>
+        <v>119.6511</v>
       </c>
       <c r="O125" s="5" t="n">
-        <v>0.3235921234165312</v>
+        <v>0.5054085040306288</v>
       </c>
     </row>
     <row r="126">
@@ -47302,10 +47314,10 @@
         <v>47.505</v>
       </c>
       <c r="N126" s="5" t="n">
-        <v>47.5875</v>
+        <v>47.7021</v>
       </c>
       <c r="O126" s="5" t="n">
-        <v>0.2878907276070332</v>
+        <v>0.5054149614120963</v>
       </c>
     </row>
     <row r="127">
@@ -47347,10 +47359,10 @@
         <v>47.741</v>
       </c>
       <c r="N127" s="5" t="n">
-        <v>47.6875</v>
+        <v>47.6562</v>
       </c>
       <c r="O127" s="5" t="n">
-        <v>0.1415465268676331</v>
+        <v>0.4856538325178467</v>
       </c>
     </row>
     <row r="128">
@@ -47392,10 +47404,10 @@
         <v>47.491</v>
       </c>
       <c r="N128" s="5" t="n">
-        <v>47.455</v>
+        <v>47.505</v>
       </c>
       <c r="O128" s="5" t="n">
-        <v>0.4309345695922442</v>
+        <v>0.4530139894804447</v>
       </c>
     </row>
     <row r="129">
@@ -47437,10 +47449,10 @@
         <v>50.005</v>
       </c>
       <c r="N129" s="5" t="n">
-        <v>49.314</v>
+        <v>49.3114</v>
       </c>
       <c r="O129" s="5" t="n">
-        <v>0.4481485987751959</v>
+        <v>0.8301506397451877</v>
       </c>
     </row>
     <row r="130">
@@ -48242,10 +48254,10 @@
         <v>3858.71</v>
       </c>
       <c r="N146" s="5" t="n">
-        <v>3886.955</v>
+        <v>3884.945</v>
       </c>
       <c r="O146" s="5" t="n">
-        <v>0.1537192995545391</v>
+        <v>0.4344962311246025</v>
       </c>
     </row>
     <row r="147">
@@ -48287,10 +48299,10 @@
         <v>3887.39</v>
       </c>
       <c r="N147" s="5" t="n">
-        <v>3876.14</v>
+        <v>3866.875</v>
       </c>
       <c r="O147" s="5" t="n">
-        <v>0.303523608538388</v>
+        <v>0.8349566707625442</v>
       </c>
     </row>
     <row r="148">
@@ -48332,10 +48344,10 @@
         <v>3891.87</v>
       </c>
       <c r="N148" s="5" t="n">
-        <v>3872.825</v>
+        <v>3869.479</v>
       </c>
       <c r="O148" s="5" t="n">
-        <v>0.5190009876511309</v>
+        <v>0.7429376992453354</v>
       </c>
     </row>
     <row r="149">
@@ -48377,10 +48389,10 @@
         <v>3863.17</v>
       </c>
       <c r="N149" s="5" t="n">
-        <v>3856.56</v>
+        <v>3857.089</v>
       </c>
       <c r="O149" s="5" t="n">
-        <v>0.2648733586408651</v>
+        <v>0.3899609511501673</v>
       </c>
     </row>
     <row r="150">
@@ -48430,10 +48442,10 @@
         <v>2145.31</v>
       </c>
       <c r="N150" s="5" t="n">
-        <v>2193.12</v>
+        <v>2257.262</v>
       </c>
       <c r="O150" s="5" t="n">
-        <v>2.834774202961983</v>
+        <v>6.276232206264939</v>
       </c>
     </row>
     <row r="151">
@@ -48475,10 +48487,10 @@
         <v>2160.76</v>
       </c>
       <c r="N151" s="5" t="n">
-        <v>2182.105</v>
+        <v>2227.31</v>
       </c>
       <c r="O151" s="5" t="n">
-        <v>2.526230405961216</v>
+        <v>5.595868664990297</v>
       </c>
     </row>
     <row r="152">
@@ -48520,10 +48532,10 @@
         <v>2162.79</v>
       </c>
       <c r="N152" s="5" t="n">
-        <v>2182.575</v>
+        <v>2233.224</v>
       </c>
       <c r="O152" s="5" t="n">
-        <v>7.095746996094054</v>
+        <v>8.051531284177472</v>
       </c>
     </row>
     <row r="153">
@@ -48565,10 +48577,10 @@
         <v>2132.5</v>
       </c>
       <c r="N153" s="5" t="n">
-        <v>2317.945</v>
+        <v>2290.043</v>
       </c>
       <c r="O153" s="5" t="n">
-        <v>5.14507462429005</v>
+        <v>5.307529262268521</v>
       </c>
     </row>
     <row r="154">
@@ -48618,10 +48630,10 @@
         <v>18327.41</v>
       </c>
       <c r="N154" s="5" t="n">
-        <v>18446.035</v>
+        <v>18095.677</v>
       </c>
       <c r="O154" s="5" t="n">
-        <v>0.4417209443655483</v>
+        <v>6.364531586430054</v>
       </c>
     </row>
     <row r="155">
@@ -48663,10 +48675,10 @@
         <v>18250.98</v>
       </c>
       <c r="N155" s="5" t="n">
-        <v>18403.695</v>
+        <v>18055.618</v>
       </c>
       <c r="O155" s="5" t="n">
-        <v>0.3751692255278088</v>
+        <v>6.344625246248723</v>
       </c>
     </row>
     <row r="156">
@@ -48708,10 +48720,10 @@
         <v>14521.54</v>
       </c>
       <c r="N156" s="5" t="n">
-        <v>17837.035</v>
+        <v>17491.973</v>
       </c>
       <c r="O156" s="5" t="n">
-        <v>0.429751917849579</v>
+        <v>6.004343048641373</v>
       </c>
     </row>
     <row r="157">
@@ -48753,10 +48765,10 @@
         <v>18033.55</v>
       </c>
       <c r="N157" s="5" t="n">
-        <v>18153.89</v>
+        <v>18195.463</v>
       </c>
       <c r="O157" s="5" t="n">
-        <v>0.302221727684809</v>
+        <v>0.8666487313711705</v>
       </c>
     </row>
     <row r="158">
@@ -48806,10 +48818,10 @@
         <v>7581.21</v>
       </c>
       <c r="N158" s="5" t="n">
-        <v>7583.57</v>
+        <v>7586.018</v>
       </c>
       <c r="O158" s="5" t="n">
-        <v>0.07621740156681088</v>
+        <v>0.1070493785933947</v>
       </c>
     </row>
     <row r="159">
@@ -48851,10 +48863,10 @@
         <v>7573.08</v>
       </c>
       <c r="N159" s="5" t="n">
-        <v>7581.21</v>
+        <v>7582.246</v>
       </c>
       <c r="O159" s="5" t="n">
-        <v>0.06779920355722012</v>
+        <v>0.1048513913392031</v>
       </c>
     </row>
     <row r="160">
@@ -48896,10 +48908,10 @@
         <v>7527.63</v>
       </c>
       <c r="N160" s="5" t="n">
-        <v>7531.014999999999</v>
+        <v>7524.202</v>
       </c>
       <c r="O160" s="5" t="n">
-        <v>0.09826032745918772</v>
+        <v>0.323137993122419</v>
       </c>
     </row>
     <row r="161">
@@ -48941,10 +48953,10 @@
         <v>6771.15</v>
       </c>
       <c r="N161" s="5" t="n">
-        <v>7562.63</v>
+        <v>7488.34</v>
       </c>
       <c r="O161" s="5" t="n">
-        <v>0.05070987209476117</v>
+        <v>3.369964262586825</v>
       </c>
     </row>
     <row r="162">
@@ -48994,10 +49006,10 @@
         <v>41816.1</v>
       </c>
       <c r="N162" s="5" t="n">
-        <v>41913.11500000001</v>
+        <v>41956.657</v>
       </c>
       <c r="O162" s="5" t="n">
-        <v>0.2499098432555036</v>
+        <v>0.4844172402805924</v>
       </c>
     </row>
     <row r="163">
@@ -49039,10 +49051,10 @@
         <v>41752.92</v>
       </c>
       <c r="N163" s="5" t="n">
-        <v>41913.1</v>
+        <v>42007.913</v>
       </c>
       <c r="O163" s="5" t="n">
-        <v>0.386609437144952</v>
+        <v>0.5429329836211321</v>
       </c>
     </row>
     <row r="164">
@@ -49084,10 +49096,10 @@
         <v>40675.56</v>
       </c>
       <c r="N164" s="5" t="n">
-        <v>40659.72</v>
+        <v>40627.002</v>
       </c>
       <c r="O164" s="5" t="n">
-        <v>0.2697632939921901</v>
+        <v>0.2758002625510442</v>
       </c>
     </row>
     <row r="165">
@@ -49129,10 +49141,10 @@
         <v>41218.04</v>
       </c>
       <c r="N165" s="5" t="n">
-        <v>41328.64999999999</v>
+        <v>41421.865</v>
       </c>
       <c r="O165" s="5" t="n">
-        <v>0.2150687235126112</v>
+        <v>0.7598814903095857</v>
       </c>
     </row>
     <row r="166">
@@ -49182,10 +49194,10 @@
         <v>48606.36</v>
       </c>
       <c r="N166" s="5" t="n">
-        <v>48602.875</v>
+        <v>48598.072</v>
       </c>
       <c r="O166" s="5" t="n">
-        <v>0.02094526301170515</v>
+        <v>0.0441296793507337</v>
       </c>
     </row>
     <row r="167">
@@ -49227,10 +49239,10 @@
         <v>48739.41</v>
       </c>
       <c r="N167" s="5" t="n">
-        <v>48766.165</v>
+        <v>48766.648</v>
       </c>
       <c r="O167" s="5" t="n">
-        <v>0.03134345298630691</v>
+        <v>0.04081719515729978</v>
       </c>
     </row>
     <row r="168">
@@ -49272,10 +49284,10 @@
         <v>48580.67</v>
       </c>
       <c r="N168" s="5" t="n">
-        <v>48602.44</v>
+        <v>48599.583</v>
       </c>
       <c r="O168" s="5" t="n">
-        <v>0.018167812150991</v>
+        <v>0.02237790810545623</v>
       </c>
     </row>
     <row r="169">
@@ -49317,10 +49329,10 @@
         <v>48590.31</v>
       </c>
       <c r="N169" s="5" t="n">
-        <v>48592.62</v>
+        <v>48586.685</v>
       </c>
       <c r="O169" s="5" t="n">
-        <v>0.02642376558415691</v>
+        <v>0.04959606020245592</v>
       </c>
     </row>
     <row r="170">
@@ -49370,10 +49382,10 @@
         <v>57344</v>
       </c>
       <c r="N170" s="5" t="n">
-        <v>57338.045</v>
+        <v>57339.609</v>
       </c>
       <c r="O170" s="5" t="n">
-        <v>0.004534511073759461</v>
+        <v>0.006491101373725714</v>
       </c>
     </row>
     <row r="171">
@@ -49415,10 +49427,10 @@
         <v>57333.56</v>
       </c>
       <c r="N171" s="5" t="n">
-        <v>57338.045</v>
+        <v>57337.668</v>
       </c>
       <c r="O171" s="5" t="n">
-        <v>0.001281871399697325</v>
+        <v>0.004596977485900014</v>
       </c>
     </row>
     <row r="172">
@@ -49460,10 +49472,10 @@
         <v>57344</v>
       </c>
       <c r="N172" s="5" t="n">
-        <v>57342.51</v>
+        <v>57340.206</v>
       </c>
       <c r="O172" s="5" t="n">
-        <v>0.001299210655409018</v>
+        <v>0.006506923345390716</v>
       </c>
     </row>
     <row r="173">
@@ -49505,10 +49517,10 @@
         <v>57337.31</v>
       </c>
       <c r="N173" s="5" t="n">
-        <v>57337.31</v>
+        <v>57336.628</v>
       </c>
       <c r="O173" s="5" t="n">
-        <v>0.002563775663701636</v>
+        <v>0.007538696728407326</v>
       </c>
     </row>
     <row r="174">
@@ -49558,10 +49570,10 @@
         <v>57454.1</v>
       </c>
       <c r="N174" s="5" t="n">
-        <v>57448.88</v>
+        <v>57450.637</v>
       </c>
       <c r="O174" s="5" t="n">
-        <v>0.003707644082873993</v>
+        <v>0.0061224318083468</v>
       </c>
     </row>
     <row r="175">
@@ -49603,10 +49615,10 @@
         <v>57446.75</v>
       </c>
       <c r="N175" s="5" t="n">
-        <v>57448.88</v>
+        <v>57447.807</v>
       </c>
       <c r="O175" s="5" t="n">
-        <v>0.004551872899874812</v>
+        <v>0.006617198716665556</v>
       </c>
     </row>
     <row r="176">
@@ -49648,10 +49660,10 @@
         <v>57443.67</v>
       </c>
       <c r="N176" s="5" t="n">
-        <v>57447.815</v>
+        <v>57446.43</v>
       </c>
       <c r="O176" s="5" t="n">
-        <v>0.004586771489920091</v>
+        <v>0.01579519031976023</v>
       </c>
     </row>
     <row r="177">
@@ -49693,10 +49705,10 @@
         <v>57451.98</v>
       </c>
       <c r="N177" s="5" t="n">
-        <v>57446.27499999999</v>
+        <v>57434.771</v>
       </c>
       <c r="O177" s="5" t="n">
-        <v>0.009931018155675059</v>
+        <v>0.0466973960414909</v>
       </c>
     </row>
     <row r="178">

</xml_diff>